<commit_message>
Add solo-developer app planning report and fix DTx reimbursement claim
New report evaluating six app concepts for the Japanese market against
the overseas research, with weighted scoring, knock-out criteria, unit
economics and revenue scenarios, an MVP spec, validation gates and
compliance guardrails. Recommends a clinician-facing case-note drafting
tool as the first product.

Correct the earlier research report (markdown and workbook): Japan does
have insured prescription digital therapeutics (e.g. Medcle, CureApp
products), so the earlier statement that no reimbursement path exists
was wrong. The conclusion that prescription DTx is out of scope for a
solo developer is unchanged.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ant9Qyu2smcXwW4HSfRnAY
</commit_message>
<xml_diff>
--- a/海外メンタルヘルスAI_未上陸サービス調査_2026.xlsx
+++ b/海外メンタルヘルスAI_未上陸サービス調査_2026.xlsx
@@ -1565,7 +1565,7 @@
       </c>
       <c r="J14" s="6" t="inlineStr">
         <is>
-          <t>FDAクリアランス＋メディケア償還モデル。日本に対応する償還経路がない</t>
+          <t>FDAクリアランス＋メディケア償還モデル。日本にも保険収載の前例（Medcle等）はあるが製品ごとの個別承認が必要</t>
         </is>
       </c>
     </row>
@@ -4071,7 +4071,7 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>メンタルヘルス領域のAI／デジタル治療について、日本に広く使われる償還経路がまだ確立していない</t>
+          <t>デジタル治療の保険収載は日本にも存在する（Medcle＝不眠障害、CureApp＝禁煙・高血圧・減酒等）。ただし製品単位で治験・薬事承認・保険収載を通す必要があり、メンタルヘルス領域の生成AIへの適用事例は確認できていない</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr"/>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>エビデンス面では最有力だが、日本に償還の受け皿がないことが決定的な制約</t>
+          <t>エビデンス面では最有力。日本にも保険収載の前例（Medcle等）はあるが、製品ごとの治験＋薬事承認＋保険収載が必要で個人・小規模開発には現実的でない</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
@@ -4432,7 +4432,7 @@
         <is>
           <t>【空白③】処方型デジタル治療
 （Big Health／HelloBetter）
-※償還経路がなく保留</t>
+※個別承認が必要で保留</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
@@ -5719,7 +5719,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5840,6 +5840,22 @@
       </c>
       <c r="D9" s="5" t="inlineStr"/>
     </row>
+    <row r="10">
+      <c r="A10" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>【訂正 2026-10-04】初版では「日本に償還の受け皿がない」と記載しましたが誤りでした</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>日本にもデジタル治療の保険収載はあります（Medcle＝不眠障害、CureApp＝禁煙・高血圧・減酒等）。ただし製品ごとの個別承認が必要で、個人・小規模開発の対象外という結論は変わりません。該当箇所は修正済み</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:C1"/>

</xml_diff>